<commit_message>
Week 8: Implement AST-based static analyzer and validate equivalence with regex engine
Added ANTLR-driven feature extraction, integrated grammar-aware detection pipeline, and implemented comparison framework demonstrating behavioral agreement between heuristic and AST analysis.

Week 8: Add comparison summary metrics for regex vs AST evaluation

Implemented automated summary generator computing agreement rate and detection totals for research evaluation.
</commit_message>
<xml_diff>
--- a/docs/weekly_deliverables.xlsx
+++ b/docs/weekly_deliverables.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Par\Documents\Old Computer Files\BCIT\1 COMP8047\QueryLens\docs\design\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Par\Documents\Old Computer Files\BCIT\1 COMP8047\QueryLens\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1399413-8429-4F47-91F1-EFAE89C58EF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9144C70F-F388-4209-AB6C-57DF85769D58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="30960" windowHeight="16800" xr2:uid="{74101E42-6690-410E-B1EF-60139AD30725}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="80">
   <si>
     <t>Week</t>
   </si>
@@ -797,6 +797,9 @@
       <c r="D6" s="2" t="s">
         <v>74</v>
       </c>
+      <c r="E6" s="2" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="2">
@@ -811,6 +814,9 @@
       <c r="D7" s="2" t="s">
         <v>77</v>
       </c>
+      <c r="E7" s="2" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="2">
@@ -825,6 +831,9 @@
       <c r="D8" s="3" t="s">
         <v>10</v>
       </c>
+      <c r="E8" s="2" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="2">
@@ -838,6 +847,9 @@
       </c>
       <c r="D9" s="3" t="s">
         <v>13</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="10" spans="1:5">

</xml_diff>

<commit_message>
Week 12: Add configurable correlation thresholds and false-positive diagnostic analysis for runtime validation
</commit_message>
<xml_diff>
--- a/docs/weekly_deliverables.xlsx
+++ b/docs/weekly_deliverables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Par\Documents\Old Computer Files\BCIT\1 COMP8047\QueryLens\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9144C70F-F388-4209-AB6C-57DF85769D58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DEEB9D3-1A01-4D95-A8BC-F7B12AE30DCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="30960" windowHeight="16800" xr2:uid="{74101E42-6690-410E-B1EF-60139AD30725}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="80">
   <si>
     <t>Week</t>
   </si>
@@ -865,6 +865,9 @@
       <c r="D10" s="3" t="s">
         <v>16</v>
       </c>
+      <c r="E10" s="2" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="2">
@@ -879,6 +882,9 @@
       <c r="D11" s="3" t="s">
         <v>19</v>
       </c>
+      <c r="E11" s="2" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="2">
@@ -892,6 +898,9 @@
       </c>
       <c r="D12" s="3" t="s">
         <v>22</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="13" spans="1:5">

</xml_diff>